<commit_message>
R41 - Findings：bsdtar+NTFS 瓶頸確認 + R41 四輪總結（2026-06-28）/ R41 - Findings: bsdtar+NTFS bottleneck confirmed + R41 full summary
- 新增 helper_windows/tar_benchmark/tar-bench-win.ps1：隔離 tar list vs extract 速度，確認 Windows decode file mode 瓶頸
- tar -tzf（list）648–844 MB/s vs tar -xzf（extract）36–174 MB/s；list/extract = 3.7×（claw）/ 23×（llama）
- LZFSE file decode（159 MB/s）≈ tar extract（174 MB/s），直接確認 bsdtar 為瓶頸，非 codec
- 新增 helper_windows/tar_benchmark/Findings.md（雙語）與 Findings_en.md（英文）
- OPTIMIZATION.md：補入 R41 總結章節，涵蓋代碼變更、四輪速度對比、Windows encode 主要發現、decode 效能摘要、RSS 峰值、R42 方向

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WAcJzuxwutWtVCWF3tcobH
</commit_message>
<xml_diff>
--- a/#trend/lzfse2_DOE_trend.xlsx
+++ b/#trend/lzfse2_DOE_trend.xlsx
@@ -8756,130 +8756,130 @@
         </is>
       </c>
       <c r="B39" s="11" t="n">
-        <v>48.73</v>
+        <v>47.47</v>
       </c>
       <c r="C39" s="11" t="n">
-        <v>375</v>
+        <v>405.51</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>344.41</v>
+        <v>348.45</v>
       </c>
       <c r="E39" s="11" t="n">
-        <v>63.73</v>
+        <v>65.08</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>34.45</v>
+        <v>34.74</v>
       </c>
       <c r="G39" s="11" t="n">
-        <v>353.65</v>
+        <v>368.84</v>
       </c>
       <c r="H39" s="11" t="n">
-        <v>394.69</v>
+        <v>418.75</v>
       </c>
       <c r="I39" s="11" t="n">
-        <v>376.09</v>
+        <v>388.48</v>
       </c>
       <c r="J39" s="11" t="n">
-        <v>326.41</v>
+        <v>273.42</v>
       </c>
       <c r="K39" s="11" t="n">
-        <v>388.52</v>
+        <v>310.67</v>
       </c>
       <c r="L39" s="11" t="n">
-        <v>365.21</v>
+        <v>332.58</v>
       </c>
       <c r="M39" s="11" t="n">
-        <v>394.7</v>
+        <v>319.62</v>
       </c>
       <c r="N39" s="11" t="n">
-        <v>422.91</v>
+        <v>422.27</v>
       </c>
       <c r="O39" s="11" t="n">
-        <v>405.75</v>
+        <v>313.11</v>
       </c>
       <c r="P39" s="11" t="n">
-        <v>4.2</v>
+        <v>4.3</v>
       </c>
       <c r="Q39" s="11" t="n">
-        <v>272.9</v>
+        <v>273.9</v>
       </c>
       <c r="R39" s="11" t="n">
-        <v>266.1</v>
+        <v>239</v>
       </c>
       <c r="S39" s="11" t="n">
-        <v>499.5</v>
+        <v>495.1</v>
       </c>
       <c r="T39" s="11" t="n">
-        <v>572.5</v>
+        <v>578.7</v>
       </c>
       <c r="U39" s="11" t="n">
-        <v>387.8</v>
+        <v>393.1</v>
       </c>
       <c r="V39" s="11" t="n">
-        <v>80.40000000000001</v>
+        <v>84.8</v>
       </c>
       <c r="W39" s="11" t="n">
         <v>3.7</v>
       </c>
       <c r="X39" s="11" t="n">
-        <v>324.5</v>
+        <v>323.4</v>
       </c>
       <c r="Y39" s="11" t="n">
-        <v>299.5</v>
+        <v>300.9</v>
       </c>
       <c r="Z39" s="11" t="n">
-        <v>320.2</v>
+        <v>320.4</v>
       </c>
       <c r="AA39" s="11" t="n">
-        <v>308.2</v>
+        <v>307.2</v>
       </c>
       <c r="AB39" s="11" t="n">
         <v>9.199999999999999</v>
       </c>
       <c r="AC39" s="11" t="n">
-        <v>33.8</v>
+        <v>33.7</v>
       </c>
       <c r="AD39" s="11" t="n">
-        <v>164.105015</v>
+        <v>183.146799</v>
       </c>
       <c r="AE39" s="11" t="n">
-        <v>29.046845</v>
+        <v>37.295865</v>
       </c>
       <c r="AF39" s="11" t="n">
-        <v>27.406304</v>
+        <v>33.195275</v>
       </c>
       <c r="AG39" s="11" t="n">
-        <v>114.589021</v>
+        <v>127.980607</v>
       </c>
       <c r="AH39" s="11" t="n">
-        <v>511.728532</v>
+        <v>516.5686940000001</v>
       </c>
       <c r="AI39" s="11" t="n">
-        <v>41.390304</v>
+        <v>48.277526</v>
       </c>
       <c r="AJ39" s="11" t="n">
-        <v>29.621507</v>
+        <v>37.848706</v>
       </c>
       <c r="AK39" s="11" t="n">
-        <v>5.824715</v>
+        <v>12.490862</v>
       </c>
       <c r="AL39" s="11" t="n">
-        <v>0.560314</v>
+        <v>7.037979</v>
       </c>
       <c r="AM39" s="11" t="n">
-        <v>0.168823</v>
+        <v>3.279762</v>
       </c>
       <c r="AN39" s="11" t="n">
-        <v>0.469074</v>
+        <v>5.675062</v>
       </c>
       <c r="AO39" s="11" t="n">
-        <v>0.456479</v>
+        <v>5.227284</v>
       </c>
       <c r="AP39" s="11" t="n">
-        <v>3.013619</v>
+        <v>7.95993</v>
       </c>
       <c r="AQ39" s="11" t="n">
-        <v>0.583399</v>
+        <v>3.653914</v>
       </c>
       <c r="AR39" s="11" t="n">
         <v>1</v>
@@ -13614,130 +13614,130 @@
         </is>
       </c>
       <c r="B39" s="11" t="n">
-        <v>39.64</v>
+        <v>42.87</v>
       </c>
       <c r="C39" s="11" t="n">
-        <v>87.88</v>
+        <v>98.34999999999999</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>86.26000000000001</v>
+        <v>98.5</v>
       </c>
       <c r="E39" s="11" t="n">
-        <v>83.84</v>
+        <v>88.78</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>49.16</v>
+        <v>51.28</v>
       </c>
       <c r="G39" s="11" t="n">
-        <v>89.91</v>
+        <v>100.3</v>
       </c>
       <c r="H39" s="11" t="n">
-        <v>85.97</v>
+        <v>95.39</v>
       </c>
       <c r="I39" s="11" t="n">
-        <v>85.66</v>
+        <v>89.75</v>
       </c>
       <c r="J39" s="11" t="n">
-        <v>78.76000000000001</v>
+        <v>79.52</v>
       </c>
       <c r="K39" s="11" t="n">
-        <v>79.31</v>
+        <v>83.86</v>
       </c>
       <c r="L39" s="11" t="n">
-        <v>79.38</v>
+        <v>85.54000000000001</v>
       </c>
       <c r="M39" s="11" t="n">
-        <v>82.06999999999999</v>
+        <v>86.39</v>
       </c>
       <c r="N39" s="11" t="n">
-        <v>82.70999999999999</v>
+        <v>84.58</v>
       </c>
       <c r="O39" s="11" t="n">
-        <v>79.78</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="P39" s="11" t="n">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="Q39" s="11" t="n">
-        <v>347.6</v>
+        <v>362.2</v>
       </c>
       <c r="R39" s="11" t="n">
-        <v>335.2</v>
+        <v>327.3</v>
       </c>
       <c r="S39" s="11" t="n">
-        <v>536.4</v>
+        <v>496.9</v>
       </c>
       <c r="T39" s="11" t="n">
-        <v>798.2</v>
+        <v>800.4</v>
       </c>
       <c r="U39" s="11" t="n">
         <v>474</v>
       </c>
       <c r="V39" s="11" t="n">
-        <v>84.5</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="W39" s="11" t="n">
         <v>3.8</v>
       </c>
       <c r="X39" s="11" t="n">
-        <v>351.2</v>
+        <v>351.3</v>
       </c>
       <c r="Y39" s="11" t="n">
-        <v>349.1</v>
+        <v>348.9</v>
       </c>
       <c r="Z39" s="11" t="n">
-        <v>348.9</v>
+        <v>348.8</v>
       </c>
       <c r="AA39" s="11" t="n">
         <v>349</v>
       </c>
       <c r="AB39" s="11" t="n">
-        <v>9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="AC39" s="11" t="n">
         <v>33.8</v>
       </c>
       <c r="AD39" s="11" t="n">
-        <v>163.996272</v>
+        <v>181.853493</v>
       </c>
       <c r="AE39" s="11" t="n">
-        <v>24.831163</v>
+        <v>38.430544</v>
       </c>
       <c r="AF39" s="11" t="n">
-        <v>21.653157</v>
+        <v>35.869722</v>
       </c>
       <c r="AG39" s="11" t="n">
-        <v>46.194363</v>
+        <v>64.052694</v>
       </c>
       <c r="AH39" s="11" t="n">
-        <v>347.988725</v>
+        <v>357.31218</v>
       </c>
       <c r="AI39" s="11" t="n">
-        <v>26.343391</v>
+        <v>31.178605</v>
       </c>
       <c r="AJ39" s="11" t="n">
-        <v>34.666265</v>
+        <v>37.862181</v>
       </c>
       <c r="AK39" s="11" t="n">
-        <v>4.876532</v>
+        <v>11.184513</v>
       </c>
       <c r="AL39" s="11" t="n">
-        <v>0.01731</v>
+        <v>2.67478</v>
       </c>
       <c r="AM39" s="11" t="n">
-        <v>0.060709</v>
+        <v>2.702654</v>
       </c>
       <c r="AN39" s="11" t="n">
-        <v>0.058143</v>
+        <v>2.433523</v>
       </c>
       <c r="AO39" s="11" t="n">
-        <v>0.13556</v>
+        <v>3.308972</v>
       </c>
       <c r="AP39" s="11" t="n">
-        <v>0.854316</v>
+        <v>4.295828</v>
       </c>
       <c r="AQ39" s="11" t="n">
-        <v>0.069609</v>
+        <v>3.19346</v>
       </c>
       <c r="AR39" s="11" t="n">
         <v>1</v>

</xml_diff>